<commit_message>
SCRUM-32: Resolve Fraud Case open decisions (Q1-Q7) and add account ID mapping
- Account ID mapping reference table (A0001/A00001/A0000001 -> A0000001) with generator, validator and tests
- Member 360: DQ-11 requires every core banking account in the mapping table
- Fraud Case: account_found_flag, SLA by priority (sla_days, sla_breached_flag), DQ-13 routing (optional),
  DQ-14 member match-rate gate, ET timezone in contract, daily status snapshot
- BREAKING: CRITICAL_CASE_AGED replaced by CASE_SLA_BREACHED; fraud_case 20 -> 23 columns
- Framework: Warehouse.replace_partition, Rule.applies; copies kept identical by test
- Unit test case documents (Member 360 130/130, Fraud Case 127/127) generated from real pytest runs
- OpenSpec change resolve-fraud-case-open-decisions and synced specs

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/DP_Fraud_Case/Data_Dictionary_Fraud_Case.xlsx
+++ b/output/DP_Fraud_Case/Data_Dictionary_Fraud_Case.xlsx
@@ -12,9 +12,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S2T_Mapping" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Source_Dictionary'!$A$1:$H$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Target_fraud_case'!$A$1:$G$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'S2T_Mapping'!$A$1:$D$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Source_Dictionary'!$A$1:$H$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Target_fraud_case'!$A$1:$G$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'S2T_Mapping'!$A$1:$D$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -643,7 +643,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Parse M/D/YYYY H:MM. Time zone not stated.</t>
+          <t>Parse M/D/YYYY H:MM. US Eastern (America/New_York), no offset.</t>
         </is>
       </c>
     </row>
@@ -985,12 +985,210 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Blank unless Closed.</t>
+          <t>Blank unless Closed. US Eastern (ET).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>account_id_map (reference)</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>source_system</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>VARCHAR(30)</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>fraud_case_mgmt</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>System the ID comes from.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>account_id_map (reference)</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>source_account_id</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Identifier</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>VARCHAR(12)</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>A0000001</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Account ID as that system writes it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>account_id_map (reference)</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>account_id</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Identifier</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>VARCHAR(10)</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr"/>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>A0000001</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Canonical ^A\d{7}$ (zero-padded: A0001, A00001 → A0000001).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>account_id_map (reference)</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>in_core_banking</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Boolean</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>BOOLEAN</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr"/>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Canonical ID exists in core banking.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>account_id_map (reference)</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>mapping_rule</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>VARCHAR(40)</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr"/>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>pad_to_7_digits</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Rule used to derive account_id.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H14"/>
+  <autoFilter ref="A1:H19"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1001,7 +1199,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1651,17 +1849,17 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>dp_load_ts</t>
+          <t>account_found_flag</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Timestamp</t>
+          <t>Boolean</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>TIMESTAMP</t>
+          <t>BOOLEAN</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1672,29 +1870,29 @@
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>YYYY-MM-DD HH:MM:SS</t>
+          <t>TRUE / FALSE</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Load time.</t>
+          <t>Account exists in core banking (via account_id_map).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>dp_batch_id</t>
+          <t>sla_days</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Identifier</t>
+          <t>Integer</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>VARCHAR(36)</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1705,17 +1903,116 @@
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="2" t="inlineStr">
         <is>
+          <t>30 / 45 / 60 / 90 by priority</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>SLA for the case priority (configurable).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>sla_breached_flag</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Boolean</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>BOOLEAN</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>TRUE / FALSE</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Elapsed days (to close, or age if open) &gt; sla_days.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>dp_load_ts</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>TIMESTAMP</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr"/>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>YYYY-MM-DD HH:MM:SS</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Load time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>dp_batch_id</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Identifier</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>VARCHAR(36)</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr"/>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
           <t>UUID</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>Pipeline run ID.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G21"/>
+  <autoFilter ref="A1:G24"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1726,7 +2023,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2156,27 +2453,93 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
+          <t>account_found_flag</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>account_id_map (fraud_case_mgmt rows)</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>in_core_banking for primary_account_id; FALSE if unmapped. Kept and reported.</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Mapped (lookup)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>sla_days</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>priority</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Settings.sla_days_by_priority[priority].</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Mapped (rule)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>sla_breached_flag</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>days_to_close / case_age_days, sla_days</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Closed: days_to_close &gt; sla_days; open: case_age_days &gt; sla_days.</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Mapped (rule)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
           <t>dp_load_ts / dp_batch_id</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>pipeline</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>Audit columns.</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>Mapped (pipeline)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D20"/>
+  <autoFilter ref="A1:D23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>